<commit_message>
implemented new PowerMeter drivers
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/calibrate/power_database.xlsx
+++ b/monet/tests/TestData/calibrate/power_database.xlsx
@@ -510,22 +510,22 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1.635047652825961e-11</v>
       </c>
       <c r="G2" t="n">
-        <v>202.2732281203495</v>
+        <v>198.8434120512646</v>
       </c>
       <c r="H2" t="n">
-        <v>99.98702555631711</v>
+        <v>100.0480175869132</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -541,22 +541,22 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>400.7705356223058</v>
+        <v>395.790939061899</v>
       </c>
       <c r="H3" t="n">
-        <v>84.96993402314307</v>
+        <v>52.5</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -572,22 +572,22 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1.101658986257803e-08</v>
+        <v>0.4726324765793626</v>
       </c>
       <c r="G4" t="n">
-        <v>998.9801898271618</v>
+        <v>998.7393007851782</v>
       </c>
       <c r="H4" t="n">
-        <v>69.9983559290999</v>
+        <v>70.03921906922076</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -605,22 +605,22 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1.754152378907747e-14</v>
       </c>
       <c r="G5" t="n">
-        <v>397.1897391582833</v>
+        <v>399.791385032008</v>
       </c>
       <c r="H5" t="n">
-        <v>54.83421197205303</v>
+        <v>55.02771787224394</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -636,22 +636,22 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4.258065144924217e-08</v>
+        <v>1.9882762103407e-11</v>
       </c>
       <c r="G6" t="n">
-        <v>1001.032367111154</v>
+        <v>1001.249734742</v>
       </c>
       <c r="H6" t="n">
-        <v>129.9829032662301</v>
+        <v>129.9599606921765</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -667,22 +667,22 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>13:54</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>9.515760179823474e-09</v>
+        <v>1.460465492578435</v>
       </c>
       <c r="G7" t="n">
-        <v>1999.880857831672</v>
+        <v>1996.454768325762</v>
       </c>
       <c r="H7" t="n">
-        <v>114.9778981368091</v>
+        <v>115.0044249666112</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -693,8 +693,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B5:B7"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ctypes wrapper for Thorlabs TLPM dll
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/calibrate/power_database.xlsx
+++ b/monet/tests/TestData/calibrate/power_database.xlsx
@@ -515,17 +515,17 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1.635047652825961e-11</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>198.8434120512646</v>
+        <v>200.859727560085</v>
       </c>
       <c r="H2" t="n">
-        <v>100.0480175869132</v>
+        <v>122.5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -546,17 +546,17 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2.047732684443819</v>
       </c>
       <c r="G3" t="n">
-        <v>395.790939061899</v>
+        <v>395.0993289006939</v>
       </c>
       <c r="H3" t="n">
-        <v>52.5</v>
+        <v>84.86231030473996</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -577,17 +577,17 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.4726324765793626</v>
+        <v>1.058684908931451</v>
       </c>
       <c r="G4" t="n">
-        <v>998.7393007851782</v>
+        <v>999.2170599014829</v>
       </c>
       <c r="H4" t="n">
-        <v>70.03921906922076</v>
+        <v>70.00033951866037</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -610,17 +610,17 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1.754152378907747e-14</v>
+        <v>1.902256130392743e-12</v>
       </c>
       <c r="G5" t="n">
-        <v>399.791385032008</v>
+        <v>400.8193052617406</v>
       </c>
       <c r="H5" t="n">
-        <v>55.02771787224394</v>
+        <v>55.05355416235386</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -641,17 +641,17 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1.9882762103407e-11</v>
+        <v>0.5929139468073217</v>
       </c>
       <c r="G6" t="n">
-        <v>1001.249734742</v>
+        <v>999.8556770193607</v>
       </c>
       <c r="H6" t="n">
-        <v>129.9599606921765</v>
+        <v>129.9471400982953</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -672,17 +672,17 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.460465492578435</v>
+        <v>6.854161682667836e-11</v>
       </c>
       <c r="G7" t="n">
-        <v>1996.454768325762</v>
+        <v>2000.733571498278</v>
       </c>
       <c r="H7" t="n">
-        <v>115.0044249666112</v>
+        <v>115.0075623930704</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cobolt Key issue fix
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/calibrate/power_database.xlsx
+++ b/monet/tests/TestData/calibrate/power_database.xlsx
@@ -515,21 +515,21 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>8.257616812556989e-12</v>
       </c>
       <c r="G2" t="n">
-        <v>200.859727560085</v>
+        <v>201.119076631117</v>
       </c>
       <c r="H2" t="n">
-        <v>122.5</v>
+        <v>99.94683157945948</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>sample</t>
         </is>
       </c>
     </row>
@@ -546,21 +546,21 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2.047732684443819</v>
+        <v>1.501072133676184</v>
       </c>
       <c r="G3" t="n">
-        <v>395.0993289006939</v>
+        <v>400.4624580097543</v>
       </c>
       <c r="H3" t="n">
-        <v>84.86231030473996</v>
+        <v>85.10692836249946</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>sample</t>
         </is>
       </c>
     </row>
@@ -577,21 +577,21 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1.058684908931451</v>
+        <v>2.488397605758394</v>
       </c>
       <c r="G4" t="n">
-        <v>999.2170599014829</v>
+        <v>997.3776765023749</v>
       </c>
       <c r="H4" t="n">
-        <v>70.00033951866037</v>
+        <v>70.02448938733519</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>sample</t>
         </is>
       </c>
     </row>
@@ -610,21 +610,21 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1.902256130392743e-12</v>
+        <v>4.690651644878585e-09</v>
       </c>
       <c r="G5" t="n">
-        <v>400.8193052617406</v>
+        <v>398.1797606259341</v>
       </c>
       <c r="H5" t="n">
-        <v>55.05355416235386</v>
+        <v>54.89512841983797</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>sample</t>
         </is>
       </c>
     </row>
@@ -641,21 +641,21 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.5929139468073217</v>
+        <v>1.983181174836091e-09</v>
       </c>
       <c r="G6" t="n">
-        <v>999.8556770193607</v>
+        <v>999.5858686360668</v>
       </c>
       <c r="H6" t="n">
-        <v>129.9471400982953</v>
+        <v>129.9891253925911</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>sample</t>
         </is>
       </c>
     </row>
@@ -672,21 +672,21 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6.854161682667836e-11</v>
+        <v>1.67829282667125</v>
       </c>
       <c r="G7" t="n">
-        <v>2000.733571498278</v>
+        <v>1999.188664684375</v>
       </c>
       <c r="H7" t="n">
-        <v>115.0075623930704</v>
+        <v>114.9532910571891</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>sample</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
switching autoshutter back on after calibration
</commit_message>
<xml_diff>
--- a/monet/tests/TestData/calibrate/power_database.xlsx
+++ b/monet/tests/TestData/calibrate/power_database.xlsx
@@ -515,17 +515,17 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8.257616812556989e-12</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>201.119076631117</v>
+        <v>199.3320068939003</v>
       </c>
       <c r="H2" t="n">
-        <v>99.94683157945948</v>
+        <v>122.5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -546,17 +546,17 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.501072133676184</v>
+        <v>1.090978619506421</v>
       </c>
       <c r="G3" t="n">
-        <v>400.4624580097543</v>
+        <v>398.3379096680424</v>
       </c>
       <c r="H3" t="n">
-        <v>85.10692836249946</v>
+        <v>84.92749003757352</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -577,17 +577,17 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2.488397605758394</v>
+        <v>6.312824485377178e-09</v>
       </c>
       <c r="G4" t="n">
-        <v>997.3776765023749</v>
+        <v>1001.383913398695</v>
       </c>
       <c r="H4" t="n">
-        <v>70.02448938733519</v>
+        <v>70.02748655449844</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -610,17 +610,17 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4.690651644878585e-09</v>
+        <v>9.25504117788023e-11</v>
       </c>
       <c r="G5" t="n">
-        <v>398.1797606259341</v>
+        <v>400.8500220421965</v>
       </c>
       <c r="H5" t="n">
-        <v>54.89512841983797</v>
+        <v>54.95169924234299</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -641,17 +641,17 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1.983181174836091e-09</v>
+        <v>1.288013448537177</v>
       </c>
       <c r="G6" t="n">
-        <v>999.5858686360668</v>
+        <v>1000.77757394131</v>
       </c>
       <c r="H6" t="n">
-        <v>129.9891253925911</v>
+        <v>130.0364062074549</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -672,17 +672,17 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.67829282667125</v>
+        <v>0.2563287750347449</v>
       </c>
       <c r="G7" t="n">
-        <v>1999.188664684375</v>
+        <v>1997.446521295876</v>
       </c>
       <c r="H7" t="n">
-        <v>114.9532910571891</v>
+        <v>115.0318488355702</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>

</xml_diff>